<commit_message>
Single login with multiple workers
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1707161580895840027'</t>
+          <t>170716158089584L8N2IN</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1</t>
+          <t>Template1_L8N2IN</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1707161580898730014'</t>
+          <t>170716158089873L8N2IN</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2</t>
+          <t>Template2_L8N2IN</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8274981748172940</t>
+          <t>82749817481L8N2IN3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3</t>
+          <t>Template3_L8N2IN</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12849821798217800</t>
+          <t>12849821798L8N2IN4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4</t>
+          <t>Template4_L8N2IN</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>812349821491874</t>
+          <t>81234982149L8N2IN5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5</t>
+          <t>Template5_L8N2IN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8274981748172940</t>
+          <t>82749817481L8N2IN6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6</t>
+          <t>Template6_L8N2IN</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12849821798217800</t>
+          <t>12849821798L8N2IN7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7</t>
+          <t>Template7_L8N2IN</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>812349821491874</t>
+          <t>81234982149L8N2IN8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8</t>
+          <t>Template8_L8N2IN</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8274981748172940</t>
+          <t>82749817481L8N2IN9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9</t>
+          <t>Template9_L8N2IN</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12849821798217800</t>
+          <t>12849821798L8N2IN10</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10</t>
+          <t>Template10_L8N2IN</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>812349821491874</t>
+          <t>81234982149L8N2IN11</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11</t>
+          <t>Template11_L8N2IN</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
sms skipped testcases updates
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>170716158089584E6N3TE</t>
+          <t>170716158089584FG0CIL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_E6N3TE</t>
+          <t>Template1_FG0CIL</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>170716158089873E6N3TE</t>
+          <t>170716158089873FG0CIL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_E6N3TE</t>
+          <t>Template2_FG0CIL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>82749817481E6N3TE3</t>
+          <t>82749817481FG0CIL3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_E6N3TE</t>
+          <t>Template3_FG0CIL</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12849821798E6N3TE4</t>
+          <t>12849821798FG0CIL4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_E6N3TE</t>
+          <t>Template4_FG0CIL</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81234982149E6N3TE5</t>
+          <t>81234982149FG0CIL5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_E6N3TE</t>
+          <t>Template5_FG0CIL</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>82749817481E6N3TE6</t>
+          <t>82749817481FG0CIL6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_E6N3TE</t>
+          <t>Template6_FG0CIL</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12849821798E6N3TE7</t>
+          <t>12849821798FG0CIL7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_E6N3TE</t>
+          <t>Template7_FG0CIL</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81234982149E6N3TE8</t>
+          <t>81234982149FG0CIL8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_E6N3TE</t>
+          <t>Template8_FG0CIL</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>82749817481E6N3TE9</t>
+          <t>82749817481FG0CIL9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_E6N3TE</t>
+          <t>Template9_FG0CIL</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12849821798E6N3TE10</t>
+          <t>12849821798FG0CIL10</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_E6N3TE</t>
+          <t>Template10_FG0CIL</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>81234982149E6N3TE11</t>
+          <t>81234982149FG0CIL11</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_E6N3TE</t>
+          <t>Template11_FG0CIL</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
export file header verification
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>170716158089584FG0CIL</t>
+          <t>170716158089584TK0N37</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_FG0CIL</t>
+          <t>Template1_TK0N37</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>170716158089873FG0CIL</t>
+          <t>170716158089873TK0N37</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_FG0CIL</t>
+          <t>Template2_TK0N37</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>82749817481FG0CIL3</t>
+          <t>82749817481TK0N373</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_FG0CIL</t>
+          <t>Template3_TK0N37</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12849821798FG0CIL4</t>
+          <t>12849821798TK0N374</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_FG0CIL</t>
+          <t>Template4_TK0N37</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81234982149FG0CIL5</t>
+          <t>81234982149TK0N375</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_FG0CIL</t>
+          <t>Template5_TK0N37</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>82749817481FG0CIL6</t>
+          <t>82749817481TK0N376</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_FG0CIL</t>
+          <t>Template6_TK0N37</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12849821798FG0CIL7</t>
+          <t>12849821798TK0N377</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_FG0CIL</t>
+          <t>Template7_TK0N37</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81234982149FG0CIL8</t>
+          <t>81234982149TK0N378</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_FG0CIL</t>
+          <t>Template8_TK0N37</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>82749817481FG0CIL9</t>
+          <t>82749817481TK0N379</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_FG0CIL</t>
+          <t>Template9_TK0N37</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12849821798FG0CIL10</t>
+          <t>12849821798TK0N3710</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_FG0CIL</t>
+          <t>Template10_TK0N37</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>81234982149FG0CIL11</t>
+          <t>81234982149TK0N3711</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_FG0CIL</t>
+          <t>Template11_TK0N37</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
Restore RCS campaign create page object (full session additions)
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>17071615808958435TQNY</t>
+          <t>170716158089584W49DF1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_35TQNY</t>
+          <t>Template1_W49DF1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>17071615808987335TQNY</t>
+          <t>170716158089873W49DF1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_35TQNY</t>
+          <t>Template2_W49DF1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8274981748135TQNY3</t>
+          <t>82749817481W49DF13</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_35TQNY</t>
+          <t>Template3_W49DF1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1284982179835TQNY4</t>
+          <t>12849821798W49DF14</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_35TQNY</t>
+          <t>Template4_W49DF1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>8123498214935TQNY5</t>
+          <t>81234982149W49DF15</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_35TQNY</t>
+          <t>Template5_W49DF1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8274981748135TQNY6</t>
+          <t>82749817481W49DF16</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_35TQNY</t>
+          <t>Template6_W49DF1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1284982179835TQNY7</t>
+          <t>12849821798W49DF17</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_35TQNY</t>
+          <t>Template7_W49DF1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>8123498214935TQNY8</t>
+          <t>81234982149W49DF18</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_35TQNY</t>
+          <t>Template8_W49DF1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8274981748135TQNY9</t>
+          <t>82749817481W49DF19</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_35TQNY</t>
+          <t>Template9_W49DF1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1284982179835TQNY10</t>
+          <t>12849821798W49DF110</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_35TQNY</t>
+          <t>Template10_W49DF1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>8123498214935TQNY11</t>
+          <t>81234982149W49DF111</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_35TQNY</t>
+          <t>Template11_W49DF1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
sms otp and rcs update
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>170716158089584NT0QJ5</t>
+          <t>170716158089584W2IGDP</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_NT0QJ5</t>
+          <t>Template1_W2IGDP</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>170716158089873NT0QJ5</t>
+          <t>170716158089873W2IGDP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_NT0QJ5</t>
+          <t>Template2_W2IGDP</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>82749817481NT0QJ53</t>
+          <t>82749817481W2IGDP3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_NT0QJ5</t>
+          <t>Template3_W2IGDP</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12849821798NT0QJ54</t>
+          <t>12849821798W2IGDP4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_NT0QJ5</t>
+          <t>Template4_W2IGDP</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81234982149NT0QJ55</t>
+          <t>81234982149W2IGDP5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_NT0QJ5</t>
+          <t>Template5_W2IGDP</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>82749817481NT0QJ56</t>
+          <t>82749817481W2IGDP6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_NT0QJ5</t>
+          <t>Template6_W2IGDP</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12849821798NT0QJ57</t>
+          <t>12849821798W2IGDP7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_NT0QJ5</t>
+          <t>Template7_W2IGDP</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81234982149NT0QJ58</t>
+          <t>81234982149W2IGDP8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_NT0QJ5</t>
+          <t>Template8_W2IGDP</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>82749817481NT0QJ59</t>
+          <t>82749817481W2IGDP9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_NT0QJ5</t>
+          <t>Template9_W2IGDP</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12849821798NT0QJ510</t>
+          <t>12849821798W2IGDP10</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_NT0QJ5</t>
+          <t>Template10_W2IGDP</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>81234982149NT0QJ511</t>
+          <t>81234982149W2IGDP11</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_NT0QJ5</t>
+          <t>Template11_W2IGDP</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
sms sender id docs update
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>170716158089584W2IGDP</t>
+          <t>170716158089584RYV8LM</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_W2IGDP</t>
+          <t>Template1_RYV8LM</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>170716158089873W2IGDP</t>
+          <t>170716158089873RYV8LM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_W2IGDP</t>
+          <t>Template2_RYV8LM</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>82749817481W2IGDP3</t>
+          <t>82749817481RYV8LM3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_W2IGDP</t>
+          <t>Template3_RYV8LM</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12849821798W2IGDP4</t>
+          <t>12849821798RYV8LM4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_W2IGDP</t>
+          <t>Template4_RYV8LM</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81234982149W2IGDP5</t>
+          <t>81234982149RYV8LM5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_W2IGDP</t>
+          <t>Template5_RYV8LM</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>82749817481W2IGDP6</t>
+          <t>82749817481RYV8LM6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_W2IGDP</t>
+          <t>Template6_RYV8LM</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12849821798W2IGDP7</t>
+          <t>12849821798RYV8LM7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_W2IGDP</t>
+          <t>Template7_RYV8LM</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81234982149W2IGDP8</t>
+          <t>81234982149RYV8LM8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_W2IGDP</t>
+          <t>Template8_RYV8LM</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>82749817481W2IGDP9</t>
+          <t>82749817481RYV8LM9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_W2IGDP</t>
+          <t>Template9_RYV8LM</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12849821798W2IGDP10</t>
+          <t>12849821798RYV8LM10</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_W2IGDP</t>
+          <t>Template10_RYV8LM</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>81234982149W2IGDP11</t>
+          <t>81234982149RYV8LM11</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_W2IGDP</t>
+          <t>Template11_RYV8LM</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
sms sender and template header update
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>170716158089584RYV8LM</t>
+          <t>170716158089584NUQH0D</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_RYV8LM</t>
+          <t>Template1_NUQH0D</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>170716158089873RYV8LM</t>
+          <t>170716158089873NUQH0D</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_RYV8LM</t>
+          <t>Template2_NUQH0D</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>82749817481RYV8LM3</t>
+          <t>82749817481NUQH0D3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_RYV8LM</t>
+          <t>Template3_NUQH0D</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12849821798RYV8LM4</t>
+          <t>12849821798NUQH0D4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_RYV8LM</t>
+          <t>Template4_NUQH0D</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81234982149RYV8LM5</t>
+          <t>81234982149NUQH0D5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_RYV8LM</t>
+          <t>Template5_NUQH0D</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>82749817481RYV8LM6</t>
+          <t>82749817481NUQH0D6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_RYV8LM</t>
+          <t>Template6_NUQH0D</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12849821798RYV8LM7</t>
+          <t>12849821798NUQH0D7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_RYV8LM</t>
+          <t>Template7_NUQH0D</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81234982149RYV8LM8</t>
+          <t>81234982149NUQH0D8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_RYV8LM</t>
+          <t>Template8_NUQH0D</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>82749817481RYV8LM9</t>
+          <t>82749817481NUQH0D9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_RYV8LM</t>
+          <t>Template9_NUQH0D</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12849821798RYV8LM10</t>
+          <t>12849821798NUQH0D10</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_RYV8LM</t>
+          <t>Template10_NUQH0D</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>81234982149RYV8LM11</t>
+          <t>81234982149NUQH0D11</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_RYV8LM</t>
+          <t>Template11_NUQH0D</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
whatsapp failed test update
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_template.xlsx
+++ b/tests/test_data/valid_template.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>170716158089584BAFXL8</t>
+          <t>170716158089584X594DT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Template1_BAFXL8</t>
+          <t>Template1_X594DT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>170716158089873BAFXL8</t>
+          <t>170716158089873X594DT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Template2_BAFXL8</t>
+          <t>Template2_X594DT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>82749817481BAFXL83</t>
+          <t>82749817481X594DT3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Template3_BAFXL8</t>
+          <t>Template3_X594DT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12849821798BAFXL84</t>
+          <t>12849821798X594DT4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Template4_BAFXL8</t>
+          <t>Template4_X594DT</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81234982149BAFXL85</t>
+          <t>81234982149X594DT5</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Template5_BAFXL8</t>
+          <t>Template5_X594DT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>82749817481BAFXL86</t>
+          <t>82749817481X594DT6</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Template6_BAFXL8</t>
+          <t>Template6_X594DT</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12849821798BAFXL87</t>
+          <t>12849821798X594DT7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Template7_BAFXL8</t>
+          <t>Template7_X594DT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81234982149BAFXL88</t>
+          <t>81234982149X594DT8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Template8_BAFXL8</t>
+          <t>Template8_X594DT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>82749817481BAFXL89</t>
+          <t>82749817481X594DT9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Template9_BAFXL8</t>
+          <t>Template9_X594DT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -817,12 +817,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12849821798BAFXL810</t>
+          <t>12849821798X594DT10</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Template10_BAFXL8</t>
+          <t>Template10_X594DT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>81234982149BAFXL811</t>
+          <t>81234982149X594DT11</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Template11_BAFXL8</t>
+          <t>Template11_X594DT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>